<commit_message>
Add harmonic column; clarify Ophiuchus's place in the framework
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143QQ9Jn3bYesJVE6qCYKuu
</commit_message>
<xml_diff>
--- a/data/Tarot-13_Master_List.xlsx
+++ b/data/Tarot-13_Master_List.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cards'!$A$5:$O$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cards'!$A$5:$P$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -139,8 +139,17 @@
       <color rgb="006B3FA0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -189,6 +198,11 @@
         <bgColor rgb="FFEEF0F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1040"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -218,7 +232,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -336,6 +350,10 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -703,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="21" min="1" max="1"/>
@@ -721,6 +739,7 @@
     <col width="22" customWidth="1" style="21" min="13" max="13"/>
     <col width="18" customWidth="1" style="21" min="14" max="14"/>
     <col width="12" customWidth="1" style="21" min="15" max="15"/>
+    <col width="18" customWidth="1" style="22" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="22">
@@ -824,6 +843,11 @@
           <t>Decan ruler</t>
         </is>
       </c>
+      <c r="P5" s="40" t="inlineStr">
+        <is>
+          <t>Harmonic</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="22">
       <c r="A6" s="28" t="n">
@@ -2105,6 +2129,11 @@
           <t>Mars</t>
         </is>
       </c>
+      <c r="P28" s="41" t="inlineStr">
+        <is>
+          <t>Conjunction (1st)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="22">
       <c r="A29" s="33" t="n">
@@ -2168,6 +2197,11 @@
           <t>Sun</t>
         </is>
       </c>
+      <c r="P29" s="41" t="inlineStr">
+        <is>
+          <t>Opposition (2nd)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="22">
       <c r="A30" s="33" t="n">
@@ -2231,6 +2265,11 @@
           <t>Jupiter</t>
         </is>
       </c>
+      <c r="P30" s="41" t="inlineStr">
+        <is>
+          <t>Trine (3rd)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="22">
       <c r="A31" s="33" t="n">
@@ -2294,6 +2333,11 @@
           <t>Sun</t>
         </is>
       </c>
+      <c r="P31" s="41" t="inlineStr">
+        <is>
+          <t>Square (4th)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="22">
       <c r="A32" s="33" t="n">
@@ -2357,6 +2401,11 @@
           <t>Jupiter</t>
         </is>
       </c>
+      <c r="P32" s="41" t="inlineStr">
+        <is>
+          <t>Quintile (5th)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="22">
       <c r="A33" s="33" t="n">
@@ -2420,6 +2469,11 @@
           <t>Mars</t>
         </is>
       </c>
+      <c r="P33" s="41" t="inlineStr">
+        <is>
+          <t>Sextile (6th)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.25" customHeight="1" s="22">
       <c r="A34" s="33" t="n">
@@ -2483,6 +2537,11 @@
           <t>Jupiter</t>
         </is>
       </c>
+      <c r="P34" s="41" t="inlineStr">
+        <is>
+          <t>Septile (7th)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="22">
       <c r="A35" s="33" t="n">
@@ -2550,6 +2609,11 @@
           <t>Mars</t>
         </is>
       </c>
+      <c r="P35" s="41" t="inlineStr">
+        <is>
+          <t>Octile (8th)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="22">
       <c r="A36" s="33" t="n">
@@ -2613,6 +2677,11 @@
           <t>Sun</t>
         </is>
       </c>
+      <c r="P36" s="41" t="inlineStr">
+        <is>
+          <t>Novile (9th)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="22">
       <c r="A37" s="33" t="n">
@@ -2959,6 +3028,11 @@
           <t>Moon</t>
         </is>
       </c>
+      <c r="P42" s="41" t="inlineStr">
+        <is>
+          <t>Conjunction (1st)</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="22">
       <c r="A43" s="35" t="n">
@@ -3022,6 +3096,11 @@
           <t>Pluto</t>
         </is>
       </c>
+      <c r="P43" s="41" t="inlineStr">
+        <is>
+          <t>Opposition (2nd)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="22">
       <c r="A44" s="35" t="n">
@@ -3085,6 +3164,11 @@
           <t>Neptune</t>
         </is>
       </c>
+      <c r="P44" s="41" t="inlineStr">
+        <is>
+          <t>Trine (3rd)</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="22">
       <c r="A45" s="35" t="n">
@@ -3148,6 +3232,11 @@
           <t>Pluto</t>
         </is>
       </c>
+      <c r="P45" s="41" t="inlineStr">
+        <is>
+          <t>Square (4th)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="23.25" customHeight="1" s="22">
       <c r="A46" s="35" t="n">
@@ -3215,6 +3304,11 @@
           <t>Neptune</t>
         </is>
       </c>
+      <c r="P46" s="41" t="inlineStr">
+        <is>
+          <t>Quintile (5th)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="22">
       <c r="A47" s="35" t="n">
@@ -3278,6 +3372,11 @@
           <t>Moon</t>
         </is>
       </c>
+      <c r="P47" s="41" t="inlineStr">
+        <is>
+          <t>Sextile (6th)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="22">
       <c r="A48" s="35" t="n">
@@ -3345,6 +3444,11 @@
           <t>Neptune</t>
         </is>
       </c>
+      <c r="P48" s="41" t="inlineStr">
+        <is>
+          <t>Septile (7th)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="22">
       <c r="A49" s="35" t="n">
@@ -3412,6 +3516,11 @@
           <t>Moon</t>
         </is>
       </c>
+      <c r="P49" s="41" t="inlineStr">
+        <is>
+          <t>Octile (8th)</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="22">
       <c r="A50" s="35" t="n">
@@ -3475,6 +3584,11 @@
           <t>Pluto</t>
         </is>
       </c>
+      <c r="P50" s="41" t="inlineStr">
+        <is>
+          <t>Novile (9th)</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="22">
       <c r="A51" s="35" t="n">
@@ -3817,6 +3931,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P56" s="41" t="inlineStr">
+        <is>
+          <t>Conjunction (1st)</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="22">
       <c r="A57" s="36" t="n">
@@ -3884,6 +4003,11 @@
           <t>Uranus</t>
         </is>
       </c>
+      <c r="P57" s="41" t="inlineStr">
+        <is>
+          <t>Opposition (2nd)</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="22">
       <c r="A58" s="36" t="n">
@@ -3947,6 +4071,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P58" s="41" t="inlineStr">
+        <is>
+          <t>Trine (3rd)</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="22">
       <c r="A59" s="36" t="n">
@@ -4010,6 +4139,11 @@
           <t>Uranus</t>
         </is>
       </c>
+      <c r="P59" s="41" t="inlineStr">
+        <is>
+          <t>Square (4th)</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="22">
       <c r="A60" s="36" t="n">
@@ -4073,6 +4207,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P60" s="41" t="inlineStr">
+        <is>
+          <t>Quintile (5th)</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="22">
       <c r="A61" s="36" t="n">
@@ -4136,6 +4275,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P61" s="41" t="inlineStr">
+        <is>
+          <t>Sextile (6th)</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="22">
       <c r="A62" s="36" t="n">
@@ -4199,6 +4343,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P62" s="41" t="inlineStr">
+        <is>
+          <t>Septile (7th)</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="22">
       <c r="A63" s="36" t="n">
@@ -4262,6 +4411,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P63" s="41" t="inlineStr">
+        <is>
+          <t>Octile (8th)</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="22">
       <c r="A64" s="36" t="n">
@@ -4325,6 +4479,11 @@
           <t>Uranus</t>
         </is>
       </c>
+      <c r="P64" s="41" t="inlineStr">
+        <is>
+          <t>Novile (9th)</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="22">
       <c r="A65" s="36" t="n">
@@ -4679,6 +4838,11 @@
           <t>Saturn</t>
         </is>
       </c>
+      <c r="P70" s="41" t="inlineStr">
+        <is>
+          <t>Conjunction (1st)</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="22">
       <c r="A71" s="38" t="n">
@@ -4742,6 +4906,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P71" s="41" t="inlineStr">
+        <is>
+          <t>Opposition (2nd)</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="22">
       <c r="A72" s="38" t="n">
@@ -4805,6 +4974,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P72" s="41" t="inlineStr">
+        <is>
+          <t>Trine (3rd)</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="22">
       <c r="A73" s="38" t="n">
@@ -4868,6 +5042,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P73" s="41" t="inlineStr">
+        <is>
+          <t>Square (4th)</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="22">
       <c r="A74" s="38" t="n">
@@ -4931,6 +5110,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P74" s="41" t="inlineStr">
+        <is>
+          <t>Quintile (5th)</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="22">
       <c r="A75" s="38" t="n">
@@ -4994,6 +5178,11 @@
           <t>Saturn</t>
         </is>
       </c>
+      <c r="P75" s="41" t="inlineStr">
+        <is>
+          <t>Sextile (6th)</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="22">
       <c r="A76" s="38" t="n">
@@ -5057,6 +5246,11 @@
           <t>Mercury</t>
         </is>
       </c>
+      <c r="P76" s="41" t="inlineStr">
+        <is>
+          <t>Septile (7th)</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="22">
       <c r="A77" s="38" t="n">
@@ -5120,6 +5314,11 @@
           <t>Saturn</t>
         </is>
       </c>
+      <c r="P77" s="41" t="inlineStr">
+        <is>
+          <t>Octile (8th)</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="23.25" customHeight="1" s="22">
       <c r="A78" s="38" t="n">
@@ -5183,6 +5382,11 @@
           <t>Venus</t>
         </is>
       </c>
+      <c r="P78" s="41" t="inlineStr">
+        <is>
+          <t>Novile (9th)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="22">
       <c r="A79" s="38" t="n">
@@ -5464,7 +5668,7 @@
       <c r="O83" s="31" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O83"/>
+  <autoFilter ref="A5:P83"/>
   <dataValidations count="1">
     <dataValidation sqref="K6:K83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Not started,Sketching,In progress,Done"</formula1>

</xml_diff>

<commit_message>
Adopt the 13-Sign Celestial Tarot spec as the deck bible
- docs/deck-bible.md: full design spec (13-sign spine, card themes, Ophiuchus language)
- Card data: themes, core lines, spec keywords, visual prompts; Page/Knight courts; The Hanged One
- Shuffler: themes on drawn cards, Five of Cups Healer card, Serpent Path spread
- README: tagline, 13-sign spine, signature card

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143QQ9Jn3bYesJVE6qCYKuu
</commit_message>
<xml_diff>
--- a/data/Tarot-13_Master_List.xlsx
+++ b/data/Tarot-13_Master_List.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cards'!$A$5:$P$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cards'!$A$5:$R$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -232,7 +232,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -354,6 +354,9 @@
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -721,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:R83"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="21" min="1" max="1"/>
@@ -740,12 +743,14 @@
     <col width="18" customWidth="1" style="21" min="14" max="14"/>
     <col width="12" customWidth="1" style="21" min="15" max="15"/>
     <col width="18" customWidth="1" style="22" min="16" max="16"/>
+    <col width="22" customWidth="1" style="22" min="17" max="17"/>
+    <col width="40" customWidth="1" style="22" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="22">
       <c r="A1" s="23" t="inlineStr">
         <is>
-          <t>Celestial Tarot — Master Card List</t>
+          <t>The 13-Sign Celestial Tarot — Master Card List</t>
         </is>
       </c>
     </row>
@@ -848,6 +853,16 @@
           <t>Harmonic</t>
         </is>
       </c>
+      <c r="Q5" s="40" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="R5" s="40" t="inlineStr">
+        <is>
+          <t>Core line</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="22">
       <c r="A6" s="28" t="n">
@@ -885,7 +900,7 @@
       </c>
       <c r="H6" s="28" t="inlineStr">
         <is>
-          <t>new beginnings, freedom, leap of faith</t>
+          <t>freedom, beginning, leap</t>
         </is>
       </c>
       <c r="I6" s="29" t="inlineStr">
@@ -911,6 +926,8 @@
       </c>
       <c r="N6" s="31" t="n"/>
       <c r="O6" s="31" t="n"/>
+      <c r="Q6" s="42" t="n"/>
+      <c r="R6" s="42" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="22">
       <c r="A7" s="28" t="n">
@@ -948,7 +965,7 @@
       </c>
       <c r="H7" s="28" t="inlineStr">
         <is>
-          <t>skill, will, communication</t>
+          <t>will, skill, manifestation</t>
         </is>
       </c>
       <c r="I7" s="29" t="n"/>
@@ -966,6 +983,8 @@
       </c>
       <c r="N7" s="31" t="n"/>
       <c r="O7" s="31" t="n"/>
+      <c r="Q7" s="42" t="n"/>
+      <c r="R7" s="42" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="22">
       <c r="A8" s="28" t="n">
@@ -1003,7 +1022,7 @@
       </c>
       <c r="H8" s="28" t="inlineStr">
         <is>
-          <t>intuition, hidden knowledge</t>
+          <t>mystery, intuition, hidden knowledge</t>
         </is>
       </c>
       <c r="I8" s="29" t="n"/>
@@ -1021,6 +1040,8 @@
       </c>
       <c r="N8" s="31" t="n"/>
       <c r="O8" s="31" t="n"/>
+      <c r="Q8" s="42" t="n"/>
+      <c r="R8" s="42" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="22">
       <c r="A9" s="28" t="n">
@@ -1058,7 +1079,7 @@
       </c>
       <c r="H9" s="28" t="inlineStr">
         <is>
-          <t>abundance, nurture, beauty</t>
+          <t>creation, fertility, abundance</t>
         </is>
       </c>
       <c r="I9" s="29" t="n"/>
@@ -1076,6 +1097,8 @@
       </c>
       <c r="N9" s="31" t="n"/>
       <c r="O9" s="31" t="n"/>
+      <c r="Q9" s="42" t="n"/>
+      <c r="R9" s="42" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="22">
       <c r="A10" s="28" t="n">
@@ -1113,7 +1136,7 @@
       </c>
       <c r="H10" s="28" t="inlineStr">
         <is>
-          <t>authority, structure, leadership</t>
+          <t>authority, initiation, sovereignty</t>
         </is>
       </c>
       <c r="I10" s="29" t="n"/>
@@ -1131,6 +1154,8 @@
       </c>
       <c r="N10" s="31" t="n"/>
       <c r="O10" s="31" t="n"/>
+      <c r="Q10" s="42" t="n"/>
+      <c r="R10" s="42" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
       <c r="A11" s="28" t="n">
@@ -1168,7 +1193,7 @@
       </c>
       <c r="H11" s="28" t="inlineStr">
         <is>
-          <t>tradition, teaching, belief</t>
+          <t>tradition, values, embodied wisdom</t>
         </is>
       </c>
       <c r="I11" s="29" t="n"/>
@@ -1186,6 +1211,8 @@
       </c>
       <c r="N11" s="31" t="n"/>
       <c r="O11" s="31" t="n"/>
+      <c r="Q11" s="42" t="n"/>
+      <c r="R11" s="42" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="22">
       <c r="A12" s="28" t="n">
@@ -1223,7 +1250,7 @@
       </c>
       <c r="H12" s="28" t="inlineStr">
         <is>
-          <t>union, choice, values</t>
+          <t>choice, union, polarity</t>
         </is>
       </c>
       <c r="I12" s="29" t="n"/>
@@ -1241,6 +1268,8 @@
       </c>
       <c r="N12" s="31" t="n"/>
       <c r="O12" s="31" t="n"/>
+      <c r="Q12" s="42" t="n"/>
+      <c r="R12" s="42" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
       <c r="A13" s="28" t="n">
@@ -1278,7 +1307,7 @@
       </c>
       <c r="H13" s="28" t="inlineStr">
         <is>
-          <t>drive, protection, victory</t>
+          <t>direction, protection, emotional will</t>
         </is>
       </c>
       <c r="I13" s="29" t="n"/>
@@ -1296,6 +1325,8 @@
       </c>
       <c r="N13" s="31" t="n"/>
       <c r="O13" s="31" t="n"/>
+      <c r="Q13" s="42" t="n"/>
+      <c r="R13" s="42" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="22">
       <c r="A14" s="28" t="n">
@@ -1333,7 +1364,7 @@
       </c>
       <c r="H14" s="28" t="inlineStr">
         <is>
-          <t>courage, inner power, patience</t>
+          <t>courage, vitality, heart</t>
         </is>
       </c>
       <c r="I14" s="29" t="n"/>
@@ -1351,6 +1382,8 @@
       </c>
       <c r="N14" s="31" t="n"/>
       <c r="O14" s="31" t="n"/>
+      <c r="Q14" s="42" t="n"/>
+      <c r="R14" s="42" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="28" t="n">
@@ -1388,7 +1421,7 @@
       </c>
       <c r="H15" s="28" t="inlineStr">
         <is>
-          <t>solitude, wisdom, inner light</t>
+          <t>discernment, solitude, inner knowledge</t>
         </is>
       </c>
       <c r="I15" s="29" t="n"/>
@@ -1406,6 +1439,8 @@
       </c>
       <c r="N15" s="31" t="n"/>
       <c r="O15" s="31" t="n"/>
+      <c r="Q15" s="42" t="n"/>
+      <c r="R15" s="42" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="22">
       <c r="A16" s="28" t="n">
@@ -1443,7 +1478,7 @@
       </c>
       <c r="H16" s="28" t="inlineStr">
         <is>
-          <t>cycles, luck, turning points</t>
+          <t>cycles, expansion, fate</t>
         </is>
       </c>
       <c r="I16" s="29" t="n"/>
@@ -1461,6 +1496,8 @@
       </c>
       <c r="N16" s="31" t="n"/>
       <c r="O16" s="31" t="n"/>
+      <c r="Q16" s="42" t="n"/>
+      <c r="R16" s="42" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="22">
       <c r="A17" s="28" t="n">
@@ -1498,7 +1535,7 @@
       </c>
       <c r="H17" s="28" t="inlineStr">
         <is>
-          <t>balance, truth, fairness</t>
+          <t>balance, truth, consequence</t>
         </is>
       </c>
       <c r="I17" s="29" t="n"/>
@@ -1516,6 +1553,8 @@
       </c>
       <c r="N17" s="31" t="n"/>
       <c r="O17" s="31" t="n"/>
+      <c r="Q17" s="42" t="n"/>
+      <c r="R17" s="42" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="22">
       <c r="A18" s="28" t="n">
@@ -1533,7 +1572,7 @@
       </c>
       <c r="D18" s="28" t="inlineStr">
         <is>
-          <t>The Hanged Man</t>
+          <t>The Hanged One</t>
         </is>
       </c>
       <c r="E18" s="28" t="inlineStr">
@@ -1553,7 +1592,7 @@
       </c>
       <c r="H18" s="28" t="inlineStr">
         <is>
-          <t>surrender, new perspective</t>
+          <t>surrender, altered perception</t>
         </is>
       </c>
       <c r="I18" s="29" t="n"/>
@@ -1571,6 +1610,8 @@
       </c>
       <c r="N18" s="31" t="n"/>
       <c r="O18" s="31" t="n"/>
+      <c r="Q18" s="42" t="n"/>
+      <c r="R18" s="42" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="22">
       <c r="A19" s="28" t="n">
@@ -1608,7 +1649,7 @@
       </c>
       <c r="H19" s="28" t="inlineStr">
         <is>
-          <t>endings, transformation</t>
+          <t>transformation, endings, rebirth</t>
         </is>
       </c>
       <c r="I19" s="29" t="n"/>
@@ -1626,6 +1667,8 @@
       </c>
       <c r="N19" s="31" t="n"/>
       <c r="O19" s="31" t="n"/>
+      <c r="Q19" s="42" t="n"/>
+      <c r="R19" s="42" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="22">
       <c r="A20" s="28" t="n">
@@ -1663,7 +1706,7 @@
       </c>
       <c r="H20" s="28" t="inlineStr">
         <is>
-          <t>moderation, blending, flow</t>
+          <t>integration, synthesis, exploration</t>
         </is>
       </c>
       <c r="I20" s="29" t="n"/>
@@ -1681,6 +1724,8 @@
       </c>
       <c r="N20" s="31" t="n"/>
       <c r="O20" s="31" t="n"/>
+      <c r="Q20" s="42" t="n"/>
+      <c r="R20" s="42" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="22">
       <c r="A21" s="28" t="n">
@@ -1718,7 +1763,7 @@
       </c>
       <c r="H21" s="28" t="inlineStr">
         <is>
-          <t>bondage, temptation, shadow</t>
+          <t>attachment, power, material bondage</t>
         </is>
       </c>
       <c r="I21" s="29" t="n"/>
@@ -1736,6 +1781,8 @@
       </c>
       <c r="N21" s="31" t="n"/>
       <c r="O21" s="31" t="n"/>
+      <c r="Q21" s="42" t="n"/>
+      <c r="R21" s="42" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="22">
       <c r="A22" s="28" t="n">
@@ -1773,7 +1820,7 @@
       </c>
       <c r="H22" s="28" t="inlineStr">
         <is>
-          <t>upheaval, sudden change</t>
+          <t>shock, rupture, liberation</t>
         </is>
       </c>
       <c r="I22" s="29" t="n"/>
@@ -1791,6 +1838,8 @@
       </c>
       <c r="N22" s="31" t="n"/>
       <c r="O22" s="31" t="n"/>
+      <c r="Q22" s="42" t="n"/>
+      <c r="R22" s="42" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="22">
       <c r="A23" s="28" t="n">
@@ -1828,7 +1877,7 @@
       </c>
       <c r="H23" s="28" t="inlineStr">
         <is>
-          <t>hope, renewal, guidance</t>
+          <t>hope, vision, collective future</t>
         </is>
       </c>
       <c r="I23" s="29" t="n"/>
@@ -1846,6 +1895,8 @@
       </c>
       <c r="N23" s="31" t="n"/>
       <c r="O23" s="31" t="n"/>
+      <c r="Q23" s="42" t="n"/>
+      <c r="R23" s="42" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="22">
       <c r="A24" s="28" t="n">
@@ -1883,7 +1934,7 @@
       </c>
       <c r="H24" s="28" t="inlineStr">
         <is>
-          <t>illusion, dreams, the unknown</t>
+          <t>dream, uncertainty, subconscious</t>
         </is>
       </c>
       <c r="I24" s="29" t="n"/>
@@ -1901,6 +1952,8 @@
       </c>
       <c r="N24" s="31" t="n"/>
       <c r="O24" s="31" t="n"/>
+      <c r="Q24" s="42" t="n"/>
+      <c r="R24" s="42" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">
       <c r="A25" s="28" t="n">
@@ -1938,7 +1991,7 @@
       </c>
       <c r="H25" s="28" t="inlineStr">
         <is>
-          <t>joy, vitality, success</t>
+          <t>life, illumination, vitality</t>
         </is>
       </c>
       <c r="I25" s="29" t="n"/>
@@ -1956,6 +2009,8 @@
       </c>
       <c r="N25" s="31" t="n"/>
       <c r="O25" s="31" t="n"/>
+      <c r="Q25" s="42" t="n"/>
+      <c r="R25" s="42" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="22">
       <c r="A26" s="28" t="n">
@@ -1973,7 +2028,7 @@
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>Judgement</t>
+          <t>Judgment</t>
         </is>
       </c>
       <c r="E26" s="28" t="inlineStr">
@@ -1993,7 +2048,7 @@
       </c>
       <c r="H26" s="28" t="inlineStr">
         <is>
-          <t>awakening, rebirth, calling</t>
+          <t>awakening, resurrection, reckoning</t>
         </is>
       </c>
       <c r="I26" s="29" t="n"/>
@@ -2011,6 +2066,8 @@
       </c>
       <c r="N26" s="31" t="n"/>
       <c r="O26" s="31" t="n"/>
+      <c r="Q26" s="42" t="n"/>
+      <c r="R26" s="42" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="22">
       <c r="A27" s="28" t="n">
@@ -2048,7 +2105,7 @@
       </c>
       <c r="H27" s="28" t="inlineStr">
         <is>
-          <t>completion, wholeness</t>
+          <t>completion, structure, wholeness</t>
         </is>
       </c>
       <c r="I27" s="29" t="n"/>
@@ -2066,6 +2123,8 @@
       </c>
       <c r="N27" s="31" t="n"/>
       <c r="O27" s="31" t="n"/>
+      <c r="Q27" s="42" t="n"/>
+      <c r="R27" s="42" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="22">
       <c r="A28" s="33" t="n">
@@ -2103,10 +2162,14 @@
       </c>
       <c r="H28" s="33" t="inlineStr">
         <is>
-          <t>seed, raw potential</t>
-        </is>
-      </c>
-      <c r="I28" s="29" t="n"/>
+          <t>beginning, desire, inspiration, initiation</t>
+        </is>
+      </c>
+      <c r="I28" s="29" t="inlineStr">
+        <is>
+          <t>Cassiopeia forming a brilliant celestial W above a newly ignited flame.</t>
+        </is>
+      </c>
       <c r="J28" s="29" t="n"/>
       <c r="K28" s="29" t="inlineStr">
         <is>
@@ -2132,6 +2195,16 @@
       <c r="P28" s="41" t="inlineStr">
         <is>
           <t>Conjunction (1st)</t>
+        </is>
+      </c>
+      <c r="Q28" s="42" t="inlineStr">
+        <is>
+          <t>Ignition</t>
+        </is>
+      </c>
+      <c r="R28" s="42" t="inlineStr">
+        <is>
+          <t>A spark becomes an intention.</t>
         </is>
       </c>
     </row>
@@ -2171,10 +2244,14 @@
       </c>
       <c r="H29" s="33" t="inlineStr">
         <is>
-          <t>duality, choice, partnership</t>
-        </is>
-      </c>
-      <c r="I29" s="29" t="n"/>
+          <t>planning, expansion, possibility, choice</t>
+        </is>
+      </c>
+      <c r="I29" s="29" t="inlineStr">
+        <is>
+          <t>A figure standing between two paths beneath Cetus.</t>
+        </is>
+      </c>
       <c r="J29" s="29" t="n"/>
       <c r="K29" s="29" t="inlineStr">
         <is>
@@ -2200,6 +2277,16 @@
       <c r="P29" s="41" t="inlineStr">
         <is>
           <t>Opposition (2nd)</t>
+        </is>
+      </c>
+      <c r="Q29" s="42" t="inlineStr">
+        <is>
+          <t>Facing the unknown</t>
+        </is>
+      </c>
+      <c r="R29" s="42" t="inlineStr">
+        <is>
+          <t>The world is larger than the territory already conquered.</t>
         </is>
       </c>
     </row>
@@ -2239,10 +2326,14 @@
       </c>
       <c r="H30" s="33" t="inlineStr">
         <is>
-          <t>growth, expression</t>
-        </is>
-      </c>
-      <c r="I30" s="29" t="n"/>
+          <t>progress, courage, expectation, movement</t>
+        </is>
+      </c>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>Perseus moving through a star field with sword raised.</t>
+        </is>
+      </c>
       <c r="J30" s="29" t="n"/>
       <c r="K30" s="29" t="inlineStr">
         <is>
@@ -2268,6 +2359,16 @@
       <c r="P30" s="41" t="inlineStr">
         <is>
           <t>Trine (3rd)</t>
+        </is>
+      </c>
+      <c r="Q30" s="42" t="inlineStr">
+        <is>
+          <t>Pursuit</t>
+        </is>
+      </c>
+      <c r="R30" s="42" t="inlineStr">
+        <is>
+          <t>Action becomes momentum.</t>
         </is>
       </c>
     </row>
@@ -2307,10 +2408,14 @@
       </c>
       <c r="H31" s="33" t="inlineStr">
         <is>
-          <t>stability, rest</t>
-        </is>
-      </c>
-      <c r="I31" s="29" t="n"/>
+          <t>celebration, home, stability, arrival</t>
+        </is>
+      </c>
+      <c r="I31" s="29" t="inlineStr">
+        <is>
+          <t>Hydra coiling around four blazing celestial pillars.</t>
+        </is>
+      </c>
       <c r="J31" s="29" t="n"/>
       <c r="K31" s="29" t="inlineStr">
         <is>
@@ -2336,6 +2441,16 @@
       <c r="P31" s="41" t="inlineStr">
         <is>
           <t>Square (4th)</t>
+        </is>
+      </c>
+      <c r="Q31" s="42" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="R31" s="42" t="inlineStr">
+        <is>
+          <t>A temporary victory becomes a place to stand.</t>
         </is>
       </c>
     </row>
@@ -2375,10 +2490,14 @@
       </c>
       <c r="H32" s="33" t="inlineStr">
         <is>
-          <t>conflict, loss, challenge</t>
-        </is>
-      </c>
-      <c r="I32" s="29" t="n"/>
+          <t>competition, tension, challenge, creative conflict</t>
+        </is>
+      </c>
+      <c r="I32" s="29" t="inlineStr">
+        <is>
+          <t>The celestial cup surrounded by competing flames.</t>
+        </is>
+      </c>
       <c r="J32" s="29" t="n"/>
       <c r="K32" s="29" t="inlineStr">
         <is>
@@ -2404,6 +2523,16 @@
       <c r="P32" s="41" t="inlineStr">
         <is>
           <t>Quintile (5th)</t>
+        </is>
+      </c>
+      <c r="Q32" s="42" t="inlineStr">
+        <is>
+          <t>Friction</t>
+        </is>
+      </c>
+      <c r="R32" s="42" t="inlineStr">
+        <is>
+          <t>Different forces collide.</t>
         </is>
       </c>
     </row>
@@ -2443,10 +2572,14 @@
       </c>
       <c r="H33" s="33" t="inlineStr">
         <is>
-          <t>harmony, exchange, recovery</t>
-        </is>
-      </c>
-      <c r="I33" s="29" t="n"/>
+          <t>victory, recognition, confidence, achievement</t>
+        </is>
+      </c>
+      <c r="I33" s="29" t="inlineStr">
+        <is>
+          <t>The raven flying above a victorious procession.</t>
+        </is>
+      </c>
       <c r="J33" s="29" t="n"/>
       <c r="K33" s="29" t="inlineStr">
         <is>
@@ -2472,6 +2605,16 @@
       <c r="P33" s="41" t="inlineStr">
         <is>
           <t>Sextile (6th)</t>
+        </is>
+      </c>
+      <c r="Q33" s="42" t="inlineStr">
+        <is>
+          <t>Recognition</t>
+        </is>
+      </c>
+      <c r="R33" s="42" t="inlineStr">
+        <is>
+          <t>The struggle produces visible results.</t>
         </is>
       </c>
     </row>
@@ -2511,10 +2654,14 @@
       </c>
       <c r="H34" s="33" t="inlineStr">
         <is>
-          <t>assessment, persistence</t>
-        </is>
-      </c>
-      <c r="I34" s="29" t="n"/>
+          <t>courage, defense, conviction, perseverance</t>
+        </is>
+      </c>
+      <c r="I34" s="29" t="inlineStr">
+        <is>
+          <t>Lyra glowing like a celestial instrument while arrows rise toward it.</t>
+        </is>
+      </c>
       <c r="J34" s="29" t="n"/>
       <c r="K34" s="29" t="inlineStr">
         <is>
@@ -2540,6 +2687,16 @@
       <c r="P34" s="41" t="inlineStr">
         <is>
           <t>Septile (7th)</t>
+        </is>
+      </c>
+      <c r="Q34" s="42" t="inlineStr">
+        <is>
+          <t>Defending the vision</t>
+        </is>
+      </c>
+      <c r="R34" s="42" t="inlineStr">
+        <is>
+          <t>Hold your position.</t>
         </is>
       </c>
     </row>
@@ -2579,10 +2736,14 @@
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
-          <t>movement, mastery, change</t>
-        </is>
-      </c>
-      <c r="I35" s="29" t="n"/>
+          <t>speed, messages, momentum, rapid change</t>
+        </is>
+      </c>
+      <c r="I35" s="29" t="inlineStr">
+        <is>
+          <t>Eight streaks of fire converging on the celestial altar.</t>
+        </is>
+      </c>
       <c r="J35" s="29" t="n"/>
       <c r="K35" s="29" t="inlineStr">
         <is>
@@ -2612,6 +2773,16 @@
       <c r="P35" s="41" t="inlineStr">
         <is>
           <t>Octile (8th)</t>
+        </is>
+      </c>
+      <c r="Q35" s="42" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="R35" s="42" t="inlineStr">
+        <is>
+          <t>Everything starts moving.</t>
         </is>
       </c>
     </row>
@@ -2651,10 +2822,14 @@
       </c>
       <c r="H36" s="33" t="inlineStr">
         <is>
-          <t>culmination, near-completion</t>
-        </is>
-      </c>
-      <c r="I36" s="29" t="n"/>
+          <t>resilience, boundaries, persistence, final effort</t>
+        </is>
+      </c>
+      <c r="I36" s="29" t="inlineStr">
+        <is>
+          <t>Draco guarding a ring of nine flames.</t>
+        </is>
+      </c>
       <c r="J36" s="29" t="n"/>
       <c r="K36" s="29" t="inlineStr">
         <is>
@@ -2680,6 +2855,16 @@
       <c r="P36" s="41" t="inlineStr">
         <is>
           <t>Novile (9th)</t>
+        </is>
+      </c>
+      <c r="Q36" s="42" t="inlineStr">
+        <is>
+          <t>Endurance</t>
+        </is>
+      </c>
+      <c r="R36" s="42" t="inlineStr">
+        <is>
+          <t>You have survived enough to know what matters.</t>
         </is>
       </c>
     </row>
@@ -2719,10 +2904,14 @@
       </c>
       <c r="H37" s="33" t="inlineStr">
         <is>
-          <t>fullness, elemental force</t>
-        </is>
-      </c>
-      <c r="I37" s="29" t="n"/>
+          <t>responsibility, overload, completion, release</t>
+        </is>
+      </c>
+      <c r="I37" s="29" t="inlineStr">
+        <is>
+          <t>Ten flames forming a heavy celestial burden.</t>
+        </is>
+      </c>
       <c r="J37" s="29" t="n"/>
       <c r="K37" s="29" t="inlineStr">
         <is>
@@ -2741,6 +2930,16 @@
       </c>
       <c r="N37" s="31" t="n"/>
       <c r="O37" s="31" t="n"/>
+      <c r="Q37" s="42" t="inlineStr">
+        <is>
+          <t>Culmination</t>
+        </is>
+      </c>
+      <c r="R37" s="42" t="inlineStr">
+        <is>
+          <t>The fire has become too much to carry.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="22">
       <c r="A38" s="33" t="n">
@@ -2753,12 +2952,12 @@
       </c>
       <c r="C38" s="33" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>Princess of Wands</t>
+          <t>Page of Wands</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr">
@@ -2768,17 +2967,17 @@
       </c>
       <c r="F38" s="33" t="inlineStr">
         <is>
-          <t>Summer Solstice</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="G38" s="33" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H38" s="33" t="inlineStr">
         <is>
-          <t>student, messenger, new energy</t>
+          <t>curiosity, adventure, experimentation</t>
         </is>
       </c>
       <c r="I38" s="29" t="n"/>
@@ -2788,7 +2987,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L38" s="33" t="n"/>
+      <c r="L38" s="33" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Princess, Summer Solstice.</t>
+        </is>
+      </c>
       <c r="M38" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -2796,6 +2999,16 @@
       </c>
       <c r="N38" s="31" t="n"/>
       <c r="O38" s="31" t="n"/>
+      <c r="Q38" s="42" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="R38" s="42" t="inlineStr">
+        <is>
+          <t>A new spark wants to explore the world.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="22">
       <c r="A39" s="33" t="n">
@@ -2808,12 +3021,12 @@
       </c>
       <c r="C39" s="33" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="D39" s="33" t="inlineStr">
         <is>
-          <t>Prince of Wands</t>
+          <t>Knight of Wands</t>
         </is>
       </c>
       <c r="E39" s="33" t="inlineStr">
@@ -2823,17 +3036,17 @@
       </c>
       <c r="F39" s="33" t="inlineStr">
         <is>
-          <t>Sagittarius</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="G39" s="33" t="inlineStr">
         <is>
-          <t>Mutable sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H39" s="33" t="inlineStr">
         <is>
-          <t>action, pursuit, movement</t>
+          <t>passion, action, risk, momentum</t>
         </is>
       </c>
       <c r="I39" s="29" t="n"/>
@@ -2843,7 +3056,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L39" s="33" t="n"/>
+      <c r="L39" s="33" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Prince, Sagittarius.</t>
+        </is>
+      </c>
       <c r="M39" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -2851,6 +3068,16 @@
       </c>
       <c r="N39" s="31" t="n"/>
       <c r="O39" s="31" t="n"/>
+      <c r="Q39" s="42" t="inlineStr">
+        <is>
+          <t>Pursuit</t>
+        </is>
+      </c>
+      <c r="R39" s="42" t="inlineStr">
+        <is>
+          <t>Fire in motion.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="22">
       <c r="A40" s="33" t="n">
@@ -2878,17 +3105,17 @@
       </c>
       <c r="F40" s="33" t="inlineStr">
         <is>
-          <t>Leo</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="G40" s="33" t="inlineStr">
         <is>
-          <t>Fixed sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H40" s="33" t="inlineStr">
         <is>
-          <t>mastery within, nurture</t>
+          <t>confidence, magnetism, creativity, independence</t>
         </is>
       </c>
       <c r="I40" s="29" t="n"/>
@@ -2898,7 +3125,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L40" s="33" t="n"/>
+      <c r="L40" s="33" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Leo (fixed sign).</t>
+        </is>
+      </c>
       <c r="M40" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -2906,6 +3137,16 @@
       </c>
       <c r="N40" s="31" t="n"/>
       <c r="O40" s="31" t="n"/>
+      <c r="Q40" s="42" t="inlineStr">
+        <is>
+          <t>Creative sovereignty</t>
+        </is>
+      </c>
+      <c r="R40" s="42" t="inlineStr">
+        <is>
+          <t>She knows what she wants and does not need permission to create it.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="22">
       <c r="A41" s="33" t="n">
@@ -2933,17 +3174,17 @@
       </c>
       <c r="F41" s="33" t="inlineStr">
         <is>
-          <t>Aries</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="G41" s="33" t="inlineStr">
         <is>
-          <t>Cardinal sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H41" s="33" t="inlineStr">
         <is>
-          <t>command, mastery without</t>
+          <t>authority, vision, courage, direction</t>
         </is>
       </c>
       <c r="I41" s="29" t="n"/>
@@ -2953,7 +3194,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L41" s="33" t="n"/>
+      <c r="L41" s="33" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Aries (cardinal sign).</t>
+        </is>
+      </c>
       <c r="M41" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -2961,6 +3206,16 @@
       </c>
       <c r="N41" s="31" t="n"/>
       <c r="O41" s="31" t="n"/>
+      <c r="Q41" s="42" t="inlineStr">
+        <is>
+          <t>Visionary command</t>
+        </is>
+      </c>
+      <c r="R41" s="42" t="inlineStr">
+        <is>
+          <t>Fire becomes leadership.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="22">
       <c r="A42" s="35" t="n">
@@ -2998,7 +3253,7 @@
       </c>
       <c r="H42" s="35" t="inlineStr">
         <is>
-          <t>seed, raw potential</t>
+          <t>opening, love, intuition, emotional birth</t>
         </is>
       </c>
       <c r="I42" s="29" t="n"/>
@@ -3033,6 +3288,16 @@
           <t>Conjunction (1st)</t>
         </is>
       </c>
+      <c r="Q42" s="42" t="inlineStr">
+        <is>
+          <t>Emotional beginning</t>
+        </is>
+      </c>
+      <c r="R42" s="42" t="inlineStr">
+        <is>
+          <t>The cup fills for the first time.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="22">
       <c r="A43" s="35" t="n">
@@ -3070,7 +3335,7 @@
       </c>
       <c r="H43" s="35" t="inlineStr">
         <is>
-          <t>duality, choice, partnership</t>
+          <t>connection, partnership, attraction, reciprocity</t>
         </is>
       </c>
       <c r="I43" s="29" t="n"/>
@@ -3101,6 +3366,16 @@
           <t>Opposition (2nd)</t>
         </is>
       </c>
+      <c r="Q43" s="42" t="inlineStr">
+        <is>
+          <t>Mutual recognition</t>
+        </is>
+      </c>
+      <c r="R43" s="42" t="inlineStr">
+        <is>
+          <t>Two beings see one another clearly.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="22">
       <c r="A44" s="35" t="n">
@@ -3138,7 +3413,7 @@
       </c>
       <c r="H44" s="35" t="inlineStr">
         <is>
-          <t>growth, expression</t>
+          <t>friendship, celebration, belonging, support</t>
         </is>
       </c>
       <c r="I44" s="29" t="n"/>
@@ -3169,6 +3444,16 @@
           <t>Trine (3rd)</t>
         </is>
       </c>
+      <c r="Q44" s="42" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="R44" s="42" t="inlineStr">
+        <is>
+          <t>Emotion becomes collective.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="22">
       <c r="A45" s="35" t="n">
@@ -3206,7 +3491,7 @@
       </c>
       <c r="H45" s="35" t="inlineStr">
         <is>
-          <t>stability, rest</t>
+          <t>contemplation, dissatisfaction, emotional retreat</t>
         </is>
       </c>
       <c r="I45" s="29" t="n"/>
@@ -3237,6 +3522,16 @@
           <t>Square (4th)</t>
         </is>
       </c>
+      <c r="Q45" s="42" t="inlineStr">
+        <is>
+          <t>Withdrawal</t>
+        </is>
+      </c>
+      <c r="R45" s="42" t="inlineStr">
+        <is>
+          <t>Something is being felt beneath the surface.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="23.25" customHeight="1" s="22">
       <c r="A46" s="35" t="n">
@@ -3274,10 +3569,14 @@
       </c>
       <c r="H46" s="35" t="inlineStr">
         <is>
-          <t>conflict, loss, challenge</t>
-        </is>
-      </c>
-      <c r="I46" s="29" t="n"/>
+          <t>healing, grief, regeneration, medicine, recovery, resurrection, transformation</t>
+        </is>
+      </c>
+      <c r="I46" s="29" t="inlineStr">
+        <is>
+          <t>A central healer holds the serpent; behind: a wounded vessel and a restored vessel, medicinal plants, a celestial staff, the Ophiuchus constellation, Scorpio descending and Sagittarius rising.</t>
+        </is>
+      </c>
       <c r="J46" s="29" t="n"/>
       <c r="K46" s="29" t="inlineStr">
         <is>
@@ -3286,7 +3585,7 @@
       </c>
       <c r="L46" s="35" t="inlineStr">
         <is>
-          <t>★ FEATURED: the 13th-sign card. 2nd decan Scorpio, decan ruler Neptune, quintile (source: Clark guidebook text, via another AI).</t>
+          <t>★ SIGNATURE CARD. Scorpio ends. Ophiuchus heals. Sagittarius rises. Upright: something damaged can be healed. Shadow: resurrecting what has completed its purpose.</t>
         </is>
       </c>
       <c r="M46" s="30" t="inlineStr">
@@ -3307,6 +3606,16 @@
       <c r="P46" s="41" t="inlineStr">
         <is>
           <t>Quintile (5th)</t>
+        </is>
+      </c>
+      <c r="Q46" s="42" t="inlineStr">
+        <is>
+          <t>Healing what was lost — THE HEALER</t>
+        </is>
+      </c>
+      <c r="R46" s="42" t="inlineStr">
+        <is>
+          <t>What was broken is not necessarily lost.</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3655,7 @@
       </c>
       <c r="H47" s="35" t="inlineStr">
         <is>
-          <t>harmony, exchange, recovery</t>
+          <t>memory, childhood, nostalgia, restoration</t>
         </is>
       </c>
       <c r="I47" s="29" t="n"/>
@@ -3377,6 +3686,16 @@
           <t>Sextile (6th)</t>
         </is>
       </c>
+      <c r="Q47" s="42" t="inlineStr">
+        <is>
+          <t>Restoration</t>
+        </is>
+      </c>
+      <c r="R47" s="42" t="inlineStr">
+        <is>
+          <t>The past returns carrying information.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="22">
       <c r="A48" s="35" t="n">
@@ -3414,7 +3733,7 @@
       </c>
       <c r="H48" s="35" t="inlineStr">
         <is>
-          <t>assessment, persistence</t>
+          <t>imagination, fantasy, options, dreams</t>
         </is>
       </c>
       <c r="I48" s="29" t="n"/>
@@ -3449,6 +3768,16 @@
           <t>Septile (7th)</t>
         </is>
       </c>
+      <c r="Q48" s="42" t="inlineStr">
+        <is>
+          <t>Possibility</t>
+        </is>
+      </c>
+      <c r="R48" s="42" t="inlineStr">
+        <is>
+          <t>Many realities appear at once.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="22">
       <c r="A49" s="35" t="n">
@@ -3486,7 +3815,7 @@
       </c>
       <c r="H49" s="35" t="inlineStr">
         <is>
-          <t>movement, mastery, change</t>
+          <t>walking away, searching, transition, spiritual journey</t>
         </is>
       </c>
       <c r="I49" s="29" t="n"/>
@@ -3521,6 +3850,16 @@
           <t>Octile (8th)</t>
         </is>
       </c>
+      <c r="Q49" s="42" t="inlineStr">
+        <is>
+          <t>Departure</t>
+        </is>
+      </c>
+      <c r="R49" s="42" t="inlineStr">
+        <is>
+          <t>Knowing when to leave.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="22">
       <c r="A50" s="35" t="n">
@@ -3558,7 +3897,7 @@
       </c>
       <c r="H50" s="35" t="inlineStr">
         <is>
-          <t>culmination, near-completion</t>
+          <t>satisfaction, pleasure, wish fulfillment, emotional reward</t>
         </is>
       </c>
       <c r="I50" s="29" t="n"/>
@@ -3589,6 +3928,16 @@
           <t>Novile (9th)</t>
         </is>
       </c>
+      <c r="Q50" s="42" t="inlineStr">
+        <is>
+          <t>Fulfillment</t>
+        </is>
+      </c>
+      <c r="R50" s="42" t="inlineStr">
+        <is>
+          <t>Desire becomes visible.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="22">
       <c r="A51" s="35" t="n">
@@ -3626,7 +3975,7 @@
       </c>
       <c r="H51" s="35" t="inlineStr">
         <is>
-          <t>fullness, elemental force</t>
+          <t>family, belonging, harmony, fulfillment</t>
         </is>
       </c>
       <c r="I51" s="29" t="n"/>
@@ -3648,6 +3997,16 @@
       </c>
       <c r="N51" s="31" t="n"/>
       <c r="O51" s="31" t="n"/>
+      <c r="Q51" s="42" t="inlineStr">
+        <is>
+          <t>Emotional wholeness</t>
+        </is>
+      </c>
+      <c r="R51" s="42" t="inlineStr">
+        <is>
+          <t>The individual becomes part of a greater emotional ecosystem.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="22">
       <c r="A52" s="35" t="n">
@@ -3660,12 +4019,12 @@
       </c>
       <c r="C52" s="35" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D52" s="35" t="inlineStr">
         <is>
-          <t>Princess of Cups</t>
+          <t>Page of Cups</t>
         </is>
       </c>
       <c r="E52" s="35" t="inlineStr">
@@ -3675,17 +4034,17 @@
       </c>
       <c r="F52" s="35" t="inlineStr">
         <is>
-          <t>Autumn Equinox</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="G52" s="35" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H52" s="35" t="inlineStr">
         <is>
-          <t>student, messenger, new energy</t>
+          <t>sensitivity, imagination, intuition</t>
         </is>
       </c>
       <c r="I52" s="29" t="n"/>
@@ -3695,7 +4054,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L52" s="35" t="n"/>
+      <c r="L52" s="35" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Princess, Autumn Equinox.</t>
+        </is>
+      </c>
       <c r="M52" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -3703,6 +4066,16 @@
       </c>
       <c r="N52" s="31" t="n"/>
       <c r="O52" s="31" t="n"/>
+      <c r="Q52" s="42" t="inlineStr">
+        <is>
+          <t>Emotional discovery</t>
+        </is>
+      </c>
+      <c r="R52" s="42" t="inlineStr">
+        <is>
+          <t>A new feeling arrives.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="22">
       <c r="A53" s="35" t="n">
@@ -3715,12 +4088,12 @@
       </c>
       <c r="C53" s="35" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="D53" s="35" t="inlineStr">
         <is>
-          <t>Prince of Cups</t>
+          <t>Knight of Cups</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
@@ -3730,17 +4103,17 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Pisces</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="G53" s="35" t="inlineStr">
         <is>
-          <t>Mutable sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H53" s="35" t="inlineStr">
         <is>
-          <t>action, pursuit, movement</t>
+          <t>romance, devotion, invitation, idealism</t>
         </is>
       </c>
       <c r="I53" s="29" t="n"/>
@@ -3750,7 +4123,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L53" s="35" t="n"/>
+      <c r="L53" s="35" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Prince, Pisces.</t>
+        </is>
+      </c>
       <c r="M53" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -3758,6 +4135,16 @@
       </c>
       <c r="N53" s="31" t="n"/>
       <c r="O53" s="31" t="n"/>
+      <c r="Q53" s="42" t="inlineStr">
+        <is>
+          <t>Emotional quest</t>
+        </is>
+      </c>
+      <c r="R53" s="42" t="inlineStr">
+        <is>
+          <t>The heart moves toward what it desires.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="22">
       <c r="A54" s="35" t="n">
@@ -3785,17 +4172,17 @@
       </c>
       <c r="F54" s="35" t="inlineStr">
         <is>
-          <t>Scorpio</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
         <is>
-          <t>Fixed sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H54" s="35" t="inlineStr">
         <is>
-          <t>mastery within, nurture</t>
+          <t>intuition, compassion, emotional intelligence</t>
         </is>
       </c>
       <c r="I54" s="29" t="n"/>
@@ -3805,7 +4192,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L54" s="35" t="n"/>
+      <c r="L54" s="35" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Scorpio (fixed sign).</t>
+        </is>
+      </c>
       <c r="M54" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -3813,6 +4204,16 @@
       </c>
       <c r="N54" s="31" t="n"/>
       <c r="O54" s="31" t="n"/>
+      <c r="Q54" s="42" t="inlineStr">
+        <is>
+          <t>Emotional sovereignty</t>
+        </is>
+      </c>
+      <c r="R54" s="42" t="inlineStr">
+        <is>
+          <t>Deep feeling without drowning in it.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="22">
       <c r="A55" s="35" t="n">
@@ -3840,17 +4241,17 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Cancer</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="G55" s="35" t="inlineStr">
         <is>
-          <t>Cardinal sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H55" s="35" t="inlineStr">
         <is>
-          <t>command, mastery without</t>
+          <t>wisdom, composure, maturity, compassion</t>
         </is>
       </c>
       <c r="I55" s="29" t="n"/>
@@ -3860,7 +4261,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L55" s="35" t="n"/>
+      <c r="L55" s="35" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Cancer (cardinal sign).</t>
+        </is>
+      </c>
       <c r="M55" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -3868,6 +4273,16 @@
       </c>
       <c r="N55" s="31" t="n"/>
       <c r="O55" s="31" t="n"/>
+      <c r="Q55" s="42" t="inlineStr">
+        <is>
+          <t>Emotional mastery</t>
+        </is>
+      </c>
+      <c r="R55" s="42" t="inlineStr">
+        <is>
+          <t>Feeling deeply while remaining centered.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="22">
       <c r="A56" s="36" t="n">
@@ -3905,7 +4320,7 @@
       </c>
       <c r="H56" s="36" t="inlineStr">
         <is>
-          <t>seed, raw potential</t>
+          <t>truth, revelation, decision, clarity</t>
         </is>
       </c>
       <c r="I56" s="29" t="n"/>
@@ -3936,6 +4351,16 @@
           <t>Conjunction (1st)</t>
         </is>
       </c>
+      <c r="Q56" s="42" t="inlineStr">
+        <is>
+          <t>Clarity</t>
+        </is>
+      </c>
+      <c r="R56" s="42" t="inlineStr">
+        <is>
+          <t>The first clean cut through confusion.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="22">
       <c r="A57" s="36" t="n">
@@ -3973,7 +4398,7 @@
       </c>
       <c r="H57" s="36" t="inlineStr">
         <is>
-          <t>duality, choice, partnership</t>
+          <t>indecision, conflict, neutrality, choice</t>
         </is>
       </c>
       <c r="I57" s="29" t="n"/>
@@ -4008,6 +4433,16 @@
           <t>Opposition (2nd)</t>
         </is>
       </c>
+      <c r="Q57" s="42" t="inlineStr">
+        <is>
+          <t>Difficult choice</t>
+        </is>
+      </c>
+      <c r="R57" s="42" t="inlineStr">
+        <is>
+          <t>Two forces pull against one another.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="22">
       <c r="A58" s="36" t="n">
@@ -4045,7 +4480,7 @@
       </c>
       <c r="H58" s="36" t="inlineStr">
         <is>
-          <t>growth, expression</t>
+          <t>grief, heartbreak, revelation, separation</t>
         </is>
       </c>
       <c r="I58" s="29" t="n"/>
@@ -4076,6 +4511,16 @@
           <t>Trine (3rd)</t>
         </is>
       </c>
+      <c r="Q58" s="42" t="inlineStr">
+        <is>
+          <t>Painful truth</t>
+        </is>
+      </c>
+      <c r="R58" s="42" t="inlineStr">
+        <is>
+          <t>The truth hurts because it changes the story.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="22">
       <c r="A59" s="36" t="n">
@@ -4113,7 +4558,7 @@
       </c>
       <c r="H59" s="36" t="inlineStr">
         <is>
-          <t>stability, rest</t>
+          <t>recovery, pause, retreat, integration</t>
         </is>
       </c>
       <c r="I59" s="29" t="n"/>
@@ -4144,6 +4589,16 @@
           <t>Square (4th)</t>
         </is>
       </c>
+      <c r="Q59" s="42" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="R59" s="42" t="inlineStr">
+        <is>
+          <t>The mind needs silence.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="22">
       <c r="A60" s="36" t="n">
@@ -4181,7 +4636,7 @@
       </c>
       <c r="H60" s="36" t="inlineStr">
         <is>
-          <t>conflict, loss, challenge</t>
+          <t>rivalry, ego, strategy, consequences</t>
         </is>
       </c>
       <c r="I60" s="29" t="n"/>
@@ -4212,6 +4667,16 @@
           <t>Quintile (5th)</t>
         </is>
       </c>
+      <c r="Q60" s="42" t="inlineStr">
+        <is>
+          <t>Conflict</t>
+        </is>
+      </c>
+      <c r="R60" s="42" t="inlineStr">
+        <is>
+          <t>Winning may not mean victory.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="22">
       <c r="A61" s="36" t="n">
@@ -4249,7 +4714,7 @@
       </c>
       <c r="H61" s="36" t="inlineStr">
         <is>
-          <t>harmony, exchange, recovery</t>
+          <t>movement, passage, recovery, transition</t>
         </is>
       </c>
       <c r="I61" s="29" t="n"/>
@@ -4280,6 +4745,16 @@
           <t>Sextile (6th)</t>
         </is>
       </c>
+      <c r="Q61" s="42" t="inlineStr">
+        <is>
+          <t>Transition</t>
+        </is>
+      </c>
+      <c r="R61" s="42" t="inlineStr">
+        <is>
+          <t>Leaving turbulence behind.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="22">
       <c r="A62" s="36" t="n">
@@ -4317,7 +4792,7 @@
       </c>
       <c r="H62" s="36" t="inlineStr">
         <is>
-          <t>assessment, persistence</t>
+          <t>strategy, secrecy, independence, cleverness</t>
         </is>
       </c>
       <c r="I62" s="29" t="n"/>
@@ -4348,6 +4823,16 @@
           <t>Septile (7th)</t>
         </is>
       </c>
+      <c r="Q62" s="42" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="R62" s="42" t="inlineStr">
+        <is>
+          <t>Not every move needs to be announced.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="22">
       <c r="A63" s="36" t="n">
@@ -4385,7 +4870,7 @@
       </c>
       <c r="H63" s="36" t="inlineStr">
         <is>
-          <t>movement, mastery, change</t>
+          <t>limitation, fear, mental loops, release</t>
         </is>
       </c>
       <c r="I63" s="29" t="n"/>
@@ -4416,6 +4901,16 @@
           <t>Octile (8th)</t>
         </is>
       </c>
+      <c r="Q63" s="42" t="inlineStr">
+        <is>
+          <t>Restriction</t>
+        </is>
+      </c>
+      <c r="R63" s="42" t="inlineStr">
+        <is>
+          <t>The cage may be partly constructed by perception.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="22">
       <c r="A64" s="36" t="n">
@@ -4453,7 +4948,7 @@
       </c>
       <c r="H64" s="36" t="inlineStr">
         <is>
-          <t>culmination, near-completion</t>
+          <t>worry, insomnia, fear, mental pressure</t>
         </is>
       </c>
       <c r="I64" s="29" t="n"/>
@@ -4484,6 +4979,16 @@
           <t>Novile (9th)</t>
         </is>
       </c>
+      <c r="Q64" s="42" t="inlineStr">
+        <is>
+          <t>Anxiety</t>
+        </is>
+      </c>
+      <c r="R64" s="42" t="inlineStr">
+        <is>
+          <t>Thought becomes its own night sky.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="22">
       <c r="A65" s="36" t="n">
@@ -4521,7 +5026,7 @@
       </c>
       <c r="H65" s="36" t="inlineStr">
         <is>
-          <t>fullness, elemental force</t>
+          <t>ending, collapse, release, finality</t>
         </is>
       </c>
       <c r="I65" s="29" t="n"/>
@@ -4543,6 +5048,16 @@
       </c>
       <c r="N65" s="31" t="n"/>
       <c r="O65" s="31" t="n"/>
+      <c r="Q65" s="42" t="inlineStr">
+        <is>
+          <t>Mental ending</t>
+        </is>
+      </c>
+      <c r="R65" s="42" t="inlineStr">
+        <is>
+          <t>The old thought-pattern has reached its limit.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="22">
       <c r="A66" s="36" t="n">
@@ -4555,12 +5070,12 @@
       </c>
       <c r="C66" s="36" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D66" s="36" t="inlineStr">
         <is>
-          <t>Princess of Swords</t>
+          <t>Page of Swords</t>
         </is>
       </c>
       <c r="E66" s="36" t="inlineStr">
@@ -4570,17 +5085,17 @@
       </c>
       <c r="F66" s="36" t="inlineStr">
         <is>
-          <t>Winter Solstice</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="G66" s="36" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H66" s="36" t="inlineStr">
         <is>
-          <t>student, messenger, new energy</t>
+          <t>curiosity, information, investigation</t>
         </is>
       </c>
       <c r="I66" s="29" t="n"/>
@@ -4590,7 +5105,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L66" s="36" t="n"/>
+      <c r="L66" s="36" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Princess, Winter Solstice.</t>
+        </is>
+      </c>
       <c r="M66" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -4598,6 +5117,16 @@
       </c>
       <c r="N66" s="31" t="n"/>
       <c r="O66" s="31" t="n"/>
+      <c r="Q66" s="42" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="R66" s="42" t="inlineStr">
+        <is>
+          <t>Question everything.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="22">
       <c r="A67" s="36" t="n">
@@ -4610,12 +5139,12 @@
       </c>
       <c r="C67" s="36" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="D67" s="36" t="inlineStr">
         <is>
-          <t>Prince of Swords</t>
+          <t>Knight of Swords</t>
         </is>
       </c>
       <c r="E67" s="36" t="inlineStr">
@@ -4625,17 +5154,17 @@
       </c>
       <c r="F67" s="36" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="G67" s="36" t="inlineStr">
         <is>
-          <t>Mutable sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H67" s="36" t="inlineStr">
         <is>
-          <t>action, pursuit, movement</t>
+          <t>speed, action, argument, determination</t>
         </is>
       </c>
       <c r="I67" s="29" t="n"/>
@@ -4645,7 +5174,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L67" s="36" t="n"/>
+      <c r="L67" s="36" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Prince, Gemini.</t>
+        </is>
+      </c>
       <c r="M67" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -4653,6 +5186,16 @@
       </c>
       <c r="N67" s="31" t="n"/>
       <c r="O67" s="31" t="n"/>
+      <c r="Q67" s="42" t="inlineStr">
+        <is>
+          <t>Decisive thought</t>
+        </is>
+      </c>
+      <c r="R67" s="42" t="inlineStr">
+        <is>
+          <t>The mind becomes an arrow.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="23.25" customHeight="1" s="22">
       <c r="A68" s="36" t="n">
@@ -4680,17 +5223,17 @@
       </c>
       <c r="F68" s="36" t="inlineStr">
         <is>
-          <t>Aquarius</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="G68" s="36" t="inlineStr">
         <is>
-          <t>Fixed sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H68" s="36" t="inlineStr">
         <is>
-          <t>mastery within, nurture</t>
+          <t>independence, truth, boundaries, intelligence</t>
         </is>
       </c>
       <c r="I68" s="29" t="n"/>
@@ -4702,7 +5245,7 @@
       </c>
       <c r="L68" s="37" t="inlineStr">
         <is>
-          <t>Fixed air. Google listed Libra (swapped); pattern says Aquarius.</t>
+          <t>Celestial Tarot original: Aquarius (fixed sign).</t>
         </is>
       </c>
       <c r="M68" s="34" t="inlineStr">
@@ -4712,6 +5255,16 @@
       </c>
       <c r="N68" s="31" t="n"/>
       <c r="O68" s="31" t="n"/>
+      <c r="Q68" s="42" t="inlineStr">
+        <is>
+          <t>Discernment</t>
+        </is>
+      </c>
+      <c r="R68" s="42" t="inlineStr">
+        <is>
+          <t>She sees through the fog.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="23.25" customHeight="1" s="22">
       <c r="A69" s="36" t="n">
@@ -4739,17 +5292,17 @@
       </c>
       <c r="F69" s="36" t="inlineStr">
         <is>
-          <t>Libra</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="G69" s="36" t="inlineStr">
         <is>
-          <t>Cardinal sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H69" s="36" t="inlineStr">
         <is>
-          <t>command, mastery without</t>
+          <t>strategy, law, reason, command</t>
         </is>
       </c>
       <c r="I69" s="29" t="n"/>
@@ -4761,7 +5314,7 @@
       </c>
       <c r="L69" s="37" t="inlineStr">
         <is>
-          <t>Cardinal air. Google listed Aquarius (swapped); pattern says Libra.</t>
+          <t>Celestial Tarot original: Libra (cardinal sign).</t>
         </is>
       </c>
       <c r="M69" s="34" t="inlineStr">
@@ -4771,6 +5324,16 @@
       </c>
       <c r="N69" s="31" t="n"/>
       <c r="O69" s="31" t="n"/>
+      <c r="Q69" s="42" t="inlineStr">
+        <is>
+          <t>Intellectual authority</t>
+        </is>
+      </c>
+      <c r="R69" s="42" t="inlineStr">
+        <is>
+          <t>Thought becomes judgment.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="23.25" customHeight="1" s="22">
       <c r="A70" s="38" t="n">
@@ -4808,7 +5371,7 @@
       </c>
       <c r="H70" s="38" t="inlineStr">
         <is>
-          <t>seed, raw potential</t>
+          <t>opportunity, money, beginning, resources</t>
         </is>
       </c>
       <c r="I70" s="29" t="n"/>
@@ -4843,6 +5406,16 @@
           <t>Conjunction (1st)</t>
         </is>
       </c>
+      <c r="Q70" s="42" t="inlineStr">
+        <is>
+          <t>Tangible opportunity</t>
+        </is>
+      </c>
+      <c r="R70" s="42" t="inlineStr">
+        <is>
+          <t>An idea becomes something real.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="22">
       <c r="A71" s="38" t="n">
@@ -4880,7 +5453,7 @@
       </c>
       <c r="H71" s="38" t="inlineStr">
         <is>
-          <t>duality, choice, partnership</t>
+          <t>adaptability, priorities, juggling, balance</t>
         </is>
       </c>
       <c r="I71" s="29" t="n"/>
@@ -4911,6 +5484,16 @@
           <t>Opposition (2nd)</t>
         </is>
       </c>
+      <c r="Q71" s="42" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+      <c r="R71" s="42" t="inlineStr">
+        <is>
+          <t>Keep everything moving without dropping yourself.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="22">
       <c r="A72" s="38" t="n">
@@ -4948,7 +5531,7 @@
       </c>
       <c r="H72" s="38" t="inlineStr">
         <is>
-          <t>growth, expression</t>
+          <t>teamwork, craftsmanship, collaboration</t>
         </is>
       </c>
       <c r="I72" s="29" t="n"/>
@@ -4979,6 +5562,16 @@
           <t>Trine (3rd)</t>
         </is>
       </c>
+      <c r="Q72" s="42" t="inlineStr">
+        <is>
+          <t>Cooperation</t>
+        </is>
+      </c>
+      <c r="R72" s="42" t="inlineStr">
+        <is>
+          <t>Skill becomes valuable when shared.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="22">
       <c r="A73" s="38" t="n">
@@ -5016,7 +5609,7 @@
       </c>
       <c r="H73" s="38" t="inlineStr">
         <is>
-          <t>stability, rest</t>
+          <t>possession, stability, control, security</t>
         </is>
       </c>
       <c r="I73" s="29" t="n"/>
@@ -5047,6 +5640,16 @@
           <t>Square (4th)</t>
         </is>
       </c>
+      <c r="Q73" s="42" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="R73" s="42" t="inlineStr">
+        <is>
+          <t>What do you hold onto, and why?</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="22">
       <c r="A74" s="38" t="n">
@@ -5084,7 +5687,7 @@
       </c>
       <c r="H74" s="38" t="inlineStr">
         <is>
-          <t>conflict, loss, challenge</t>
+          <t>scarcity, exclusion, survival, endurance</t>
         </is>
       </c>
       <c r="I74" s="29" t="n"/>
@@ -5115,6 +5718,16 @@
           <t>Quintile (5th)</t>
         </is>
       </c>
+      <c r="Q74" s="42" t="inlineStr">
+        <is>
+          <t>Hardship</t>
+        </is>
+      </c>
+      <c r="R74" s="42" t="inlineStr">
+        <is>
+          <t>Material difficulty tests resilience.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="22">
       <c r="A75" s="38" t="n">
@@ -5152,7 +5765,7 @@
       </c>
       <c r="H75" s="38" t="inlineStr">
         <is>
-          <t>harmony, exchange, recovery</t>
+          <t>generosity, reciprocity, support, fairness</t>
         </is>
       </c>
       <c r="I75" s="29" t="n"/>
@@ -5183,6 +5796,16 @@
           <t>Sextile (6th)</t>
         </is>
       </c>
+      <c r="Q75" s="42" t="inlineStr">
+        <is>
+          <t>Exchange</t>
+        </is>
+      </c>
+      <c r="R75" s="42" t="inlineStr">
+        <is>
+          <t>Resources move between people.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="22">
       <c r="A76" s="38" t="n">
@@ -5220,7 +5843,7 @@
       </c>
       <c r="H76" s="38" t="inlineStr">
         <is>
-          <t>assessment, persistence</t>
+          <t>patience, assessment, investment, waiting</t>
         </is>
       </c>
       <c r="I76" s="29" t="n"/>
@@ -5251,6 +5874,16 @@
           <t>Septile (7th)</t>
         </is>
       </c>
+      <c r="Q76" s="42" t="inlineStr">
+        <is>
+          <t>Cultivation</t>
+        </is>
+      </c>
+      <c r="R76" s="42" t="inlineStr">
+        <is>
+          <t>Not everything grows on your preferred schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="22">
       <c r="A77" s="38" t="n">
@@ -5288,7 +5921,7 @@
       </c>
       <c r="H77" s="38" t="inlineStr">
         <is>
-          <t>movement, mastery, change</t>
+          <t>work, skill, apprenticeship, mastery</t>
         </is>
       </c>
       <c r="I77" s="29" t="n"/>
@@ -5319,6 +5952,16 @@
           <t>Octile (8th)</t>
         </is>
       </c>
+      <c r="Q77" s="42" t="inlineStr">
+        <is>
+          <t>Mastery</t>
+        </is>
+      </c>
+      <c r="R77" s="42" t="inlineStr">
+        <is>
+          <t>Practice turns effort into craft.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="23.25" customHeight="1" s="22">
       <c r="A78" s="38" t="n">
@@ -5356,7 +5999,7 @@
       </c>
       <c r="H78" s="38" t="inlineStr">
         <is>
-          <t>culmination, near-completion</t>
+          <t>independence, harvest, self-sufficiency, accomplishment</t>
         </is>
       </c>
       <c r="I78" s="29" t="n"/>
@@ -5387,6 +6030,16 @@
           <t>Novile (9th)</t>
         </is>
       </c>
+      <c r="Q78" s="42" t="inlineStr">
+        <is>
+          <t>Independence</t>
+        </is>
+      </c>
+      <c r="R78" s="42" t="inlineStr">
+        <is>
+          <t>You built something capable of sustaining you.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="22">
       <c r="A79" s="38" t="n">
@@ -5424,7 +6077,7 @@
       </c>
       <c r="H79" s="38" t="inlineStr">
         <is>
-          <t>fullness, elemental force</t>
+          <t>family, inheritance, continuity, long-term security</t>
         </is>
       </c>
       <c r="I79" s="29" t="n"/>
@@ -5446,6 +6099,16 @@
       </c>
       <c r="N79" s="31" t="n"/>
       <c r="O79" s="31" t="n"/>
+      <c r="Q79" s="42" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="R79" s="42" t="inlineStr">
+        <is>
+          <t>What survives you?</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="22">
       <c r="A80" s="38" t="n">
@@ -5458,12 +6121,12 @@
       </c>
       <c r="C80" s="38" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D80" s="38" t="inlineStr">
         <is>
-          <t>Princess of Pentacles</t>
+          <t>Page of Pentacles</t>
         </is>
       </c>
       <c r="E80" s="38" t="inlineStr">
@@ -5473,17 +6136,17 @@
       </c>
       <c r="F80" s="38" t="inlineStr">
         <is>
-          <t>Spring Equinox</t>
+          <t>Earth</t>
         </is>
       </c>
       <c r="G80" s="38" t="inlineStr">
         <is>
-          <t>Season</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H80" s="38" t="inlineStr">
         <is>
-          <t>student, messenger, new energy</t>
+          <t>learning, opportunity, study, potential</t>
         </is>
       </c>
       <c r="I80" s="29" t="n"/>
@@ -5493,7 +6156,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L80" s="38" t="n"/>
+      <c r="L80" s="38" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Princess, Spring Equinox.</t>
+        </is>
+      </c>
       <c r="M80" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -5501,6 +6168,16 @@
       </c>
       <c r="N80" s="31" t="n"/>
       <c r="O80" s="31" t="n"/>
+      <c r="Q80" s="42" t="inlineStr">
+        <is>
+          <t>Practical beginning</t>
+        </is>
+      </c>
+      <c r="R80" s="42" t="inlineStr">
+        <is>
+          <t>A student discovers something worth building.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="22">
       <c r="A81" s="38" t="n">
@@ -5513,12 +6190,12 @@
       </c>
       <c r="C81" s="38" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="D81" s="38" t="inlineStr">
         <is>
-          <t>Prince of Pentacles</t>
+          <t>Knight of Pentacles</t>
         </is>
       </c>
       <c r="E81" s="38" t="inlineStr">
@@ -5528,17 +6205,17 @@
       </c>
       <c r="F81" s="38" t="inlineStr">
         <is>
-          <t>Virgo</t>
+          <t>Earth</t>
         </is>
       </c>
       <c r="G81" s="38" t="inlineStr">
         <is>
-          <t>Mutable sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H81" s="38" t="inlineStr">
         <is>
-          <t>action, pursuit, movement</t>
+          <t>reliability, patience, work, consistency</t>
         </is>
       </c>
       <c r="I81" s="29" t="n"/>
@@ -5548,7 +6225,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L81" s="38" t="n"/>
+      <c r="L81" s="38" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Prince, Virgo.</t>
+        </is>
+      </c>
       <c r="M81" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -5556,6 +6237,16 @@
       </c>
       <c r="N81" s="31" t="n"/>
       <c r="O81" s="31" t="n"/>
+      <c r="Q81" s="42" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="R81" s="42" t="inlineStr">
+        <is>
+          <t>Slow is not the same as stagnant.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="22">
       <c r="A82" s="38" t="n">
@@ -5583,17 +6274,17 @@
       </c>
       <c r="F82" s="38" t="inlineStr">
         <is>
-          <t>Taurus</t>
+          <t>Earth</t>
         </is>
       </c>
       <c r="G82" s="38" t="inlineStr">
         <is>
-          <t>Fixed sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H82" s="38" t="inlineStr">
         <is>
-          <t>mastery within, nurture</t>
+          <t>nourishment, abundance, practicality, care</t>
         </is>
       </c>
       <c r="I82" s="29" t="n"/>
@@ -5603,7 +6294,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L82" s="38" t="n"/>
+      <c r="L82" s="38" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Taurus (fixed sign).</t>
+        </is>
+      </c>
       <c r="M82" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -5611,6 +6306,16 @@
       </c>
       <c r="N82" s="31" t="n"/>
       <c r="O82" s="31" t="n"/>
+      <c r="Q82" s="42" t="inlineStr">
+        <is>
+          <t>Grounded abundance</t>
+        </is>
+      </c>
+      <c r="R82" s="42" t="inlineStr">
+        <is>
+          <t>She creates environments in which life can flourish.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="22">
       <c r="A83" s="38" t="n">
@@ -5638,17 +6343,17 @@
       </c>
       <c r="F83" s="38" t="inlineStr">
         <is>
-          <t>Capricorn</t>
+          <t>Earth</t>
         </is>
       </c>
       <c r="G83" s="38" t="inlineStr">
         <is>
-          <t>Cardinal sign</t>
+          <t>Element</t>
         </is>
       </c>
       <c r="H83" s="38" t="inlineStr">
         <is>
-          <t>command, mastery without</t>
+          <t>stability, leadership, prosperity, mastery</t>
         </is>
       </c>
       <c r="I83" s="29" t="n"/>
@@ -5658,7 +6363,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L83" s="38" t="n"/>
+      <c r="L83" s="38" t="inlineStr">
+        <is>
+          <t>Celestial Tarot original: Capricorn (cardinal sign).</t>
+        </is>
+      </c>
       <c r="M83" s="32" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -5666,9 +6375,19 @@
       </c>
       <c r="N83" s="31" t="n"/>
       <c r="O83" s="31" t="n"/>
+      <c r="Q83" s="42" t="inlineStr">
+        <is>
+          <t>Stewardship</t>
+        </is>
+      </c>
+      <c r="R83" s="42" t="inlineStr">
+        <is>
+          <t>Resources become responsibility.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:P83"/>
+  <autoFilter ref="A5:R83"/>
   <dataValidations count="1">
     <dataValidation sqref="K6:K83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Not started,Sketching,In progress,Done"</formula1>

</xml_diff>

<commit_message>
Make Tarot 13 upright-only: remove all reversal logic
- Remove reversal toggle, card flipping in wash/cut, reversed display, counter and rules
- Every card has one core meaning (core_meaning; new lines for the 22 Majors)
- Reading resolves each card's aspect (constructive, challenging, blocked,
  excessive, internal, warning) from the question, position and neighbors
- Add question field, aspect labels and the upright-only explanation
- Update README, deck bible, spreads guide, style guide and card data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143QQ9Jn3bYesJVE6qCYKuu
</commit_message>
<xml_diff>
--- a/data/Tarot-13_Master_List.xlsx
+++ b/data/Tarot-13_Master_List.xlsx
@@ -757,7 +757,7 @@
     <row r="2" ht="15" customHeight="1" s="22">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>Fill in the yellow columns (Art direction, Palette, Status). Row 1 (The Fool) shows an example. Correspondences from Google AI screenshots, partly corrected from Brian Clark's own text (see Source check column); keywords are general tarot meanings.</t>
+          <t>Upright-only deck: every card has one core meaning (column R). Fill in the yellow columns. Correspondences per the Source check column.</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="R5" s="40" t="inlineStr">
         <is>
-          <t>Core line</t>
+          <t>Core meaning</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,11 @@
       <c r="N6" s="31" t="n"/>
       <c r="O6" s="31" t="n"/>
       <c r="Q6" s="42" t="n"/>
-      <c r="R6" s="42" t="n"/>
+      <c r="R6" s="42" t="inlineStr">
+        <is>
+          <t>A leap into the unknown with open hands.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="22">
       <c r="A7" s="28" t="n">
@@ -984,7 +988,11 @@
       <c r="N7" s="31" t="n"/>
       <c r="O7" s="31" t="n"/>
       <c r="Q7" s="42" t="n"/>
-      <c r="R7" s="42" t="n"/>
+      <c r="R7" s="42" t="inlineStr">
+        <is>
+          <t>Will and skill focused into deliberate creation.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="22">
       <c r="A8" s="28" t="n">
@@ -1041,7 +1049,11 @@
       <c r="N8" s="31" t="n"/>
       <c r="O8" s="31" t="n"/>
       <c r="Q8" s="42" t="n"/>
-      <c r="R8" s="42" t="n"/>
+      <c r="R8" s="42" t="inlineStr">
+        <is>
+          <t>Hidden knowledge that speaks through intuition and silence.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="22">
       <c r="A9" s="28" t="n">
@@ -1098,7 +1110,11 @@
       <c r="N9" s="31" t="n"/>
       <c r="O9" s="31" t="n"/>
       <c r="Q9" s="42" t="n"/>
-      <c r="R9" s="42" t="n"/>
+      <c r="R9" s="42" t="inlineStr">
+        <is>
+          <t>Creative abundance that grows when it is nurtured.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="22">
       <c r="A10" s="28" t="n">
@@ -1155,7 +1171,11 @@
       <c r="N10" s="31" t="n"/>
       <c r="O10" s="31" t="n"/>
       <c r="Q10" s="42" t="n"/>
-      <c r="R10" s="42" t="n"/>
+      <c r="R10" s="42" t="inlineStr">
+        <is>
+          <t>Structure and authority that give life a firm shape.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
       <c r="A11" s="28" t="n">
@@ -1212,7 +1232,11 @@
       <c r="N11" s="31" t="n"/>
       <c r="O11" s="31" t="n"/>
       <c r="Q11" s="42" t="n"/>
-      <c r="R11" s="42" t="n"/>
+      <c r="R11" s="42" t="inlineStr">
+        <is>
+          <t>Tradition and shared values as a teacher.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="22">
       <c r="A12" s="28" t="n">
@@ -1269,7 +1293,11 @@
       <c r="N12" s="31" t="n"/>
       <c r="O12" s="31" t="n"/>
       <c r="Q12" s="42" t="n"/>
-      <c r="R12" s="42" t="n"/>
+      <c r="R12" s="42" t="inlineStr">
+        <is>
+          <t>A meaningful choice that reveals what you truly value.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
       <c r="A13" s="28" t="n">
@@ -1326,7 +1354,11 @@
       <c r="N13" s="31" t="n"/>
       <c r="O13" s="31" t="n"/>
       <c r="Q13" s="42" t="n"/>
-      <c r="R13" s="42" t="n"/>
+      <c r="R13" s="42" t="inlineStr">
+        <is>
+          <t>Emotional will steering toward a chosen direction.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="22">
       <c r="A14" s="28" t="n">
@@ -1383,7 +1415,11 @@
       <c r="N14" s="31" t="n"/>
       <c r="O14" s="31" t="n"/>
       <c r="Q14" s="42" t="n"/>
-      <c r="R14" s="42" t="n"/>
+      <c r="R14" s="42" t="inlineStr">
+        <is>
+          <t>Courage of the heart that wins through patience, not force.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="28" t="n">
@@ -1440,7 +1476,11 @@
       <c r="N15" s="31" t="n"/>
       <c r="O15" s="31" t="n"/>
       <c r="Q15" s="42" t="n"/>
-      <c r="R15" s="42" t="n"/>
+      <c r="R15" s="42" t="inlineStr">
+        <is>
+          <t>Solitude and discernment that light the inner path.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="22">
       <c r="A16" s="28" t="n">
@@ -1497,7 +1537,11 @@
       <c r="N16" s="31" t="n"/>
       <c r="O16" s="31" t="n"/>
       <c r="Q16" s="42" t="n"/>
-      <c r="R16" s="42" t="n"/>
+      <c r="R16" s="42" t="inlineStr">
+        <is>
+          <t>The turning of cycles, luck and timing beyond your control.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="22">
       <c r="A17" s="28" t="n">
@@ -1554,7 +1598,11 @@
       <c r="N17" s="31" t="n"/>
       <c r="O17" s="31" t="n"/>
       <c r="Q17" s="42" t="n"/>
-      <c r="R17" s="42" t="n"/>
+      <c r="R17" s="42" t="inlineStr">
+        <is>
+          <t>Truth, balance and the consequences of action.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="22">
       <c r="A18" s="28" t="n">
@@ -1611,7 +1659,11 @@
       <c r="N18" s="31" t="n"/>
       <c r="O18" s="31" t="n"/>
       <c r="Q18" s="42" t="n"/>
-      <c r="R18" s="42" t="n"/>
+      <c r="R18" s="42" t="inlineStr">
+        <is>
+          <t>Surrender that brings a new way of seeing.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="22">
       <c r="A19" s="28" t="n">
@@ -1668,7 +1720,11 @@
       <c r="N19" s="31" t="n"/>
       <c r="O19" s="31" t="n"/>
       <c r="Q19" s="42" t="n"/>
-      <c r="R19" s="42" t="n"/>
+      <c r="R19" s="42" t="inlineStr">
+        <is>
+          <t>An ending that clears the ground for transformation.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="22">
       <c r="A20" s="28" t="n">
@@ -1725,7 +1781,11 @@
       <c r="N20" s="31" t="n"/>
       <c r="O20" s="31" t="n"/>
       <c r="Q20" s="42" t="n"/>
-      <c r="R20" s="42" t="n"/>
+      <c r="R20" s="42" t="inlineStr">
+        <is>
+          <t>Blending opposites into a workable whole.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="22">
       <c r="A21" s="28" t="n">
@@ -1782,7 +1842,11 @@
       <c r="N21" s="31" t="n"/>
       <c r="O21" s="31" t="n"/>
       <c r="Q21" s="42" t="n"/>
-      <c r="R21" s="42" t="n"/>
+      <c r="R21" s="42" t="inlineStr">
+        <is>
+          <t>Attachments and appetites that bind or empower.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="22">
       <c r="A22" s="28" t="n">
@@ -1839,7 +1903,11 @@
       <c r="N22" s="31" t="n"/>
       <c r="O22" s="31" t="n"/>
       <c r="Q22" s="42" t="n"/>
-      <c r="R22" s="42" t="n"/>
+      <c r="R22" s="42" t="inlineStr">
+        <is>
+          <t>Sudden rupture that breaks what was false.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="22">
       <c r="A23" s="28" t="n">
@@ -1896,7 +1964,11 @@
       <c r="N23" s="31" t="n"/>
       <c r="O23" s="31" t="n"/>
       <c r="Q23" s="42" t="n"/>
-      <c r="R23" s="42" t="n"/>
+      <c r="R23" s="42" t="inlineStr">
+        <is>
+          <t>Hope and vision renewed after the storm.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="22">
       <c r="A24" s="28" t="n">
@@ -1953,7 +2025,11 @@
       <c r="N24" s="31" t="n"/>
       <c r="O24" s="31" t="n"/>
       <c r="Q24" s="42" t="n"/>
-      <c r="R24" s="42" t="n"/>
+      <c r="R24" s="42" t="inlineStr">
+        <is>
+          <t>Dreams, uncertainty and what moves beneath the surface.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">
       <c r="A25" s="28" t="n">
@@ -2010,7 +2086,11 @@
       <c r="N25" s="31" t="n"/>
       <c r="O25" s="31" t="n"/>
       <c r="Q25" s="42" t="n"/>
-      <c r="R25" s="42" t="n"/>
+      <c r="R25" s="42" t="inlineStr">
+        <is>
+          <t>Clarity, vitality and joy in full light.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="22">
       <c r="A26" s="28" t="n">
@@ -2067,7 +2147,11 @@
       <c r="N26" s="31" t="n"/>
       <c r="O26" s="31" t="n"/>
       <c r="Q26" s="42" t="n"/>
-      <c r="R26" s="42" t="n"/>
+      <c r="R26" s="42" t="inlineStr">
+        <is>
+          <t>An awakening call to rise and answer.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="22">
       <c r="A27" s="28" t="n">
@@ -2124,7 +2208,11 @@
       <c r="N27" s="31" t="n"/>
       <c r="O27" s="31" t="n"/>
       <c r="Q27" s="42" t="n"/>
-      <c r="R27" s="42" t="n"/>
+      <c r="R27" s="42" t="inlineStr">
+        <is>
+          <t>Completion, wholeness and the end of a great cycle.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="22">
       <c r="A28" s="33" t="n">
@@ -3585,7 +3673,7 @@
       </c>
       <c r="L46" s="35" t="inlineStr">
         <is>
-          <t>★ SIGNATURE CARD. Scorpio ends. Ophiuchus heals. Sagittarius rises. Upright: something damaged can be healed. Shadow: resurrecting what has completed its purpose.</t>
+          <t>★ SIGNATURE CARD. Scorpio ends. Ophiuchus heals. Sagittarius rises. Constructive expression: something damaged can be healed. Challenging expression: trying to resurrect what has completed its purpose.</t>
         </is>
       </c>
       <c r="M46" s="30" t="inlineStr">

</xml_diff>